<commit_message>
added new data for Adm. Tribunales
</commit_message>
<xml_diff>
--- a/data/administracion_de_tribunales/OP_148_SoliGrupEdad.xlsx
+++ b/data/administracion_de_tribunales/OP_148_SoliGrupEdad.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\administracion_de_tribunales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782F101C-349F-4D77-A86E-921C931ED71E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C8C03B9-0B17-4667-9860-986704A4D575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" tabRatio="828" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" tabRatio="828" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020-2021" sheetId="4" r:id="rId1"/>
@@ -479,6 +479,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="2">
+        <f>SUM(C2:I2)</f>
         <v>12</v>
       </c>
       <c r="C2" s="2">
@@ -502,6 +503,7 @@
         <v>10</v>
       </c>
       <c r="B3" s="2">
+        <f t="shared" ref="B3:B11" si="0">SUM(C3:I3)</f>
         <v>3</v>
       </c>
       <c r="C3" s="2">
@@ -519,6 +521,7 @@
         <v>11</v>
       </c>
       <c r="B4" s="2">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C4" s="2">
@@ -542,6 +545,7 @@
         <v>12</v>
       </c>
       <c r="B5" s="2">
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="C5" s="2">
@@ -565,6 +569,7 @@
         <v>13</v>
       </c>
       <c r="B6" s="2">
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C6" s="2">
@@ -588,6 +593,7 @@
         <v>14</v>
       </c>
       <c r="B7" s="2">
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C7" s="2">
@@ -605,6 +611,7 @@
         <v>15</v>
       </c>
       <c r="B8" s="2">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C8" s="2">
@@ -625,6 +632,7 @@
         <v>16</v>
       </c>
       <c r="B9" s="2">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C9" s="2">
@@ -639,6 +647,7 @@
         <v>17</v>
       </c>
       <c r="B10" s="2">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C10" s="2">
@@ -656,6 +665,7 @@
         <v>18</v>
       </c>
       <c r="B11" s="2">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H11" s="2">
@@ -667,35 +677,35 @@
         <v>1</v>
       </c>
       <c r="B12">
-        <f t="shared" ref="B12:I12" si="0">SUM(B2:B11)</f>
+        <f t="shared" ref="B12:I12" si="1">SUM(B2:B11)</f>
         <v>134</v>
       </c>
       <c r="C12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>79</v>
       </c>
       <c r="D12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="E12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="F12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="G12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="H12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="I12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
@@ -747,6 +757,7 @@
         <v>9</v>
       </c>
       <c r="B2">
+        <f>SUM(C2:I2)</f>
         <v>21</v>
       </c>
       <c r="C2">
@@ -767,6 +778,7 @@
         <v>10</v>
       </c>
       <c r="B3">
+        <f t="shared" ref="B3:B13" si="0">SUM(C3:I3)</f>
         <v>4</v>
       </c>
       <c r="C3">
@@ -781,6 +793,7 @@
         <v>11</v>
       </c>
       <c r="B4">
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C4">
@@ -801,6 +814,7 @@
         <v>12</v>
       </c>
       <c r="B5">
+        <f t="shared" si="0"/>
         <v>67</v>
       </c>
       <c r="C5">
@@ -830,6 +844,7 @@
         <v>13</v>
       </c>
       <c r="B6">
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C6">
@@ -859,6 +874,7 @@
         <v>14</v>
       </c>
       <c r="B7">
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C7">
@@ -885,6 +901,7 @@
         <v>15</v>
       </c>
       <c r="B8">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C8">
@@ -905,6 +922,7 @@
         <v>16</v>
       </c>
       <c r="B9">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C9">
@@ -922,6 +940,7 @@
         <v>17</v>
       </c>
       <c r="B10">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C10">
@@ -942,6 +961,7 @@
         <v>18</v>
       </c>
       <c r="B11">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C11">
@@ -959,6 +979,7 @@
         <v>19</v>
       </c>
       <c r="B12">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C12">
@@ -982,6 +1003,7 @@
         <v>20</v>
       </c>
       <c r="B13">
+        <f t="shared" si="0"/>
         <v>41</v>
       </c>
       <c r="C13">
@@ -1011,6 +1033,7 @@
         <v>21</v>
       </c>
       <c r="B14">
+        <f>SUM(C14:I14)</f>
         <v>8</v>
       </c>
       <c r="C14">
@@ -1025,35 +1048,35 @@
         <v>1</v>
       </c>
       <c r="B15">
-        <f t="shared" ref="B15:I15" si="0">SUM(B2:B14)</f>
+        <f t="shared" ref="B15:I15" si="1">SUM(B2:B14)</f>
         <v>261</v>
       </c>
       <c r="C15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>144</v>
       </c>
       <c r="D15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
       <c r="E15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="F15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="G15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="H15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>29</v>
       </c>
     </row>
@@ -1110,6 +1133,7 @@
         <v>9</v>
       </c>
       <c r="B2">
+        <f>SUM(C2:I2)</f>
         <v>5</v>
       </c>
       <c r="C2">
@@ -1127,6 +1151,7 @@
         <v>10</v>
       </c>
       <c r="B3">
+        <f t="shared" ref="B3:B14" si="0">SUM(C3:I3)</f>
         <v>5</v>
       </c>
       <c r="C3">
@@ -1144,6 +1169,7 @@
         <v>11</v>
       </c>
       <c r="B4">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C4">
@@ -1161,6 +1187,7 @@
         <v>12</v>
       </c>
       <c r="B5">
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
       <c r="C5">
@@ -1184,6 +1211,7 @@
         <v>13</v>
       </c>
       <c r="B6">
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C6">
@@ -1207,6 +1235,7 @@
         <v>14</v>
       </c>
       <c r="B7">
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C7">
@@ -1227,6 +1256,7 @@
         <v>15</v>
       </c>
       <c r="B8">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C8">
@@ -1247,6 +1277,7 @@
         <v>16</v>
       </c>
       <c r="B9">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C9">
@@ -1267,6 +1298,7 @@
         <v>17</v>
       </c>
       <c r="B10">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C10">
@@ -1284,6 +1316,7 @@
         <v>18</v>
       </c>
       <c r="B11">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C11">
@@ -1298,6 +1331,7 @@
         <v>19</v>
       </c>
       <c r="B12">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C12">
@@ -1324,6 +1358,7 @@
         <v>20</v>
       </c>
       <c r="B13">
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C13">
@@ -1353,6 +1388,7 @@
         <v>21</v>
       </c>
       <c r="B14">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C14">
@@ -1377,27 +1413,27 @@
         <v>196</v>
       </c>
       <c r="C15">
-        <f t="shared" ref="C15:I15" si="0">SUM(C2:C14)</f>
+        <f t="shared" ref="C15:H15" si="1">SUM(C2:C14)</f>
         <v>118</v>
       </c>
       <c r="D15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="E15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="F15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="G15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="H15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I15">
@@ -1456,6 +1492,7 @@
         <v>9</v>
       </c>
       <c r="B2">
+        <f>SUM(C2:I2)</f>
         <v>19</v>
       </c>
       <c r="C2">
@@ -1479,6 +1516,7 @@
         <v>10</v>
       </c>
       <c r="B3">
+        <f t="shared" ref="B3:B14" si="0">SUM(C3:I3)</f>
         <v>9</v>
       </c>
       <c r="C3">
@@ -1496,6 +1534,7 @@
         <v>11</v>
       </c>
       <c r="B4">
+        <f t="shared" si="0"/>
         <v>36</v>
       </c>
       <c r="C4">
@@ -1522,6 +1561,7 @@
         <v>12</v>
       </c>
       <c r="B5">
+        <f t="shared" si="0"/>
         <v>79</v>
       </c>
       <c r="C5">
@@ -1545,6 +1585,7 @@
         <v>13</v>
       </c>
       <c r="B6">
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C6">
@@ -1571,6 +1612,7 @@
         <v>14</v>
       </c>
       <c r="B7">
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C7">
@@ -1597,6 +1639,7 @@
         <v>15</v>
       </c>
       <c r="B8">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C8">
@@ -1620,6 +1663,7 @@
         <v>16</v>
       </c>
       <c r="B9">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C9">
@@ -1643,6 +1687,7 @@
         <v>17</v>
       </c>
       <c r="B10">
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C10">
@@ -1666,6 +1711,7 @@
         <v>18</v>
       </c>
       <c r="B11">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C11">
@@ -1677,6 +1723,7 @@
         <v>19</v>
       </c>
       <c r="B12">
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C12">
@@ -1700,6 +1747,7 @@
         <v>20</v>
       </c>
       <c r="B13">
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
       <c r="C13">
@@ -1729,6 +1777,7 @@
         <v>21</v>
       </c>
       <c r="B14">
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C14">
@@ -1756,31 +1805,31 @@
         <v>333</v>
       </c>
       <c r="C15">
-        <f t="shared" ref="C15:I15" si="0">SUM(C2:C14)</f>
+        <f t="shared" ref="C15:I15" si="1">SUM(C2:C14)</f>
         <v>183</v>
       </c>
       <c r="D15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>32</v>
       </c>
       <c r="E15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="F15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
       <c r="G15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="H15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="I15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>68</v>
       </c>
     </row>
@@ -1835,6 +1884,7 @@
         <v>9</v>
       </c>
       <c r="B2">
+        <f>SUM(C2:I2)</f>
         <v>21</v>
       </c>
       <c r="C2">
@@ -1864,6 +1914,7 @@
         <v>10</v>
       </c>
       <c r="B3">
+        <f t="shared" ref="B3:B14" si="0">SUM(C3:I3)</f>
         <v>11</v>
       </c>
       <c r="C3">
@@ -1893,6 +1944,7 @@
         <v>11</v>
       </c>
       <c r="B4">
+        <f t="shared" si="0"/>
         <v>44</v>
       </c>
       <c r="C4">
@@ -1922,6 +1974,7 @@
         <v>12</v>
       </c>
       <c r="B5">
+        <f t="shared" si="0"/>
         <v>80</v>
       </c>
       <c r="C5">
@@ -1951,6 +2004,7 @@
         <v>13</v>
       </c>
       <c r="B6">
+        <f t="shared" si="0"/>
         <v>47</v>
       </c>
       <c r="C6">
@@ -1980,6 +2034,7 @@
         <v>14</v>
       </c>
       <c r="B7">
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C7">
@@ -2009,6 +2064,7 @@
         <v>15</v>
       </c>
       <c r="B8">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C8">
@@ -2038,6 +2094,7 @@
         <v>16</v>
       </c>
       <c r="B9">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C9">
@@ -2067,6 +2124,7 @@
         <v>17</v>
       </c>
       <c r="B10">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C10">
@@ -2096,6 +2154,7 @@
         <v>18</v>
       </c>
       <c r="B11">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C11">
@@ -2125,6 +2184,7 @@
         <v>19</v>
       </c>
       <c r="B12">
+        <f t="shared" si="0"/>
         <v>44</v>
       </c>
       <c r="C12">
@@ -2154,6 +2214,7 @@
         <v>20</v>
       </c>
       <c r="B13">
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
       <c r="C13">
@@ -2183,6 +2244,7 @@
         <v>21</v>
       </c>
       <c r="B14">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C14">
@@ -2216,31 +2278,31 @@
         <v>372</v>
       </c>
       <c r="C15">
-        <f t="shared" ref="C15:I15" si="0">SUM(C2:C14)</f>
+        <f t="shared" ref="C15:I15" si="1">SUM(C2:C14)</f>
         <v>184</v>
       </c>
       <c r="D15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>41</v>
       </c>
       <c r="E15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="F15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="G15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="H15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="I15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>94</v>
       </c>
     </row>
@@ -2295,25 +2357,26 @@
         <v>9</v>
       </c>
       <c r="B2">
-        <v>12</v>
+        <f>SUM(C2:I2)</f>
+        <v>39</v>
       </c>
       <c r="C2">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I2">
         <v>1</v>
@@ -2324,19 +2387,20 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <f t="shared" ref="B3:B14" si="0">SUM(C3:I3)</f>
+        <v>14</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -2345,7 +2409,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -2353,25 +2417,26 @@
         <v>11</v>
       </c>
       <c r="B4">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="C4">
         <v>14</v>
       </c>
-      <c r="C4">
-        <v>5</v>
-      </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F4">
         <v>2</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I4">
         <v>3</v>
@@ -2382,28 +2447,29 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>44</v>
+        <f t="shared" si="0"/>
+        <v>82</v>
       </c>
       <c r="C5">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="D5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E5">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I5">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -2411,28 +2477,29 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>20</v>
+        <f t="shared" si="0"/>
+        <v>44</v>
       </c>
       <c r="C6">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -2440,28 +2507,29 @@
         <v>14</v>
       </c>
       <c r="B7">
-        <v>23</v>
+        <f t="shared" si="0"/>
+        <v>49</v>
       </c>
       <c r="C7">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -2469,28 +2537,29 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>6</v>
+        <f t="shared" si="0"/>
+        <v>17</v>
       </c>
       <c r="C8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H8">
         <v>0</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -2498,25 +2567,26 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>12</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F9">
         <v>1</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -2527,16 +2597,17 @@
         <v>17</v>
       </c>
       <c r="B10">
-        <v>4</v>
+        <f t="shared" si="0"/>
+        <v>12</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -2545,7 +2616,7 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -2556,13 +2627,14 @@
         <v>18</v>
       </c>
       <c r="B11">
-        <v>4</v>
+        <f t="shared" si="0"/>
+        <v>13</v>
       </c>
       <c r="C11">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -2571,10 +2643,10 @@
         <v>0</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11">
         <v>1</v>
@@ -2585,16 +2657,17 @@
         <v>19</v>
       </c>
       <c r="B12">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="C12">
         <v>16</v>
       </c>
-      <c r="C12">
-        <v>14</v>
-      </c>
       <c r="D12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12">
         <v>2</v>
@@ -2603,7 +2676,7 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I12">
         <v>0</v>
@@ -2614,28 +2687,29 @@
         <v>20</v>
       </c>
       <c r="B13">
-        <v>23</v>
+        <f t="shared" si="0"/>
+        <v>64</v>
       </c>
       <c r="C13">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="D13">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E13">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F13">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H13">
         <v>1</v>
       </c>
       <c r="I13">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -2643,10 +2717,11 @@
         <v>21</v>
       </c>
       <c r="B14">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>9</v>
       </c>
       <c r="C14">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -2664,7 +2739,7 @@
         <v>0</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
@@ -2673,35 +2748,35 @@
       </c>
       <c r="B15">
         <f>SUM(B2:B14)</f>
-        <v>179</v>
+        <v>405</v>
       </c>
       <c r="C15">
-        <f t="shared" ref="C15:I15" si="0">SUM(C2:C14)</f>
-        <v>108</v>
+        <f t="shared" ref="C15:I15" si="1">SUM(C2:C14)</f>
+        <v>218</v>
       </c>
       <c r="D15">
-        <f t="shared" si="0"/>
-        <v>14</v>
+        <f t="shared" si="1"/>
+        <v>38</v>
       </c>
       <c r="E15">
-        <f t="shared" si="0"/>
-        <v>19</v>
+        <f t="shared" si="1"/>
+        <v>55</v>
       </c>
       <c r="F15">
-        <f t="shared" si="0"/>
-        <v>13</v>
+        <f t="shared" si="1"/>
+        <v>45</v>
       </c>
       <c r="G15">
-        <f t="shared" si="0"/>
-        <v>6</v>
+        <f t="shared" si="1"/>
+        <v>16</v>
       </c>
       <c r="H15">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f t="shared" si="1"/>
+        <v>17</v>
       </c>
       <c r="I15">
-        <f t="shared" si="0"/>
-        <v>15</v>
+        <f t="shared" si="1"/>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>